<commit_message>
feat: :sparkles: modulo-mis-palmeras | modulo-reportes: Mejoras + configuración
</commit_message>
<xml_diff>
--- a/ceia-proyecto-final/modulo-IA/notebooks/deteccion_picudo_rojo/yolov11/entrenamientos_hiperparametros.xlsx
+++ b/ceia-proyecto-final/modulo-IA/notebooks/deteccion_picudo_rojo/yolov11/entrenamientos_hiperparametros.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Git Repositories\uba-ceia-proy-final\ceia-proyecto-final\modulo-IA\notebooks\deteccion_picudo_rojo\yolov11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6969C61D-5064-428F-88B6-4A11D2DDB78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12E697D-8C40-47EE-969F-66070F7C16E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B6CA6A92-4DAC-4216-81F7-6D0831CFCD0F}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{B6CA6A92-4DAC-4216-81F7-6D0831CFCD0F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="5" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="21">
   <si>
     <t>auto</t>
   </si>
@@ -494,31 +494,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BAC84E6-D505-4458-8AD5-88508E041B54}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="5"/>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5"/>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="1">
+        <v>2</v>
+      </c>
+      <c r="F2" s="1">
+        <v>3</v>
+      </c>
+      <c r="G2" s="1">
+        <v>4</v>
+      </c>
+      <c r="H2" s="1">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -531,8 +550,14 @@
       <c r="D3" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="1">
         <v>2</v>
@@ -541,8 +566,15 @@
         <v>13</v>
       </c>
       <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="1">
         <v>3</v>
@@ -551,8 +583,13 @@
         <v>14</v>
       </c>
       <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="H5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="1">
         <v>4</v>
@@ -561,8 +598,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="I6" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
@@ -575,8 +617,23 @@
       <c r="D7" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="1">
         <v>6</v>
@@ -585,8 +642,10 @@
         <v>1</v>
       </c>
       <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
@@ -597,8 +656,10 @@
         <v>0.01</v>
       </c>
       <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="1">
         <v>8</v>
@@ -607,8 +668,10 @@
         <v>1E-3</v>
       </c>
       <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>5</v>
       </c>
@@ -619,8 +682,10 @@
         <v>0.1</v>
       </c>
       <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="1">
         <v>10</v>
@@ -629,8 +694,10 @@
         <v>0.01</v>
       </c>
       <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>6</v>
       </c>
@@ -641,8 +708,10 @@
         <v>5</v>
       </c>
       <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="1">
         <v>12</v>
@@ -653,8 +722,23 @@
       <c r="D14" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
       <c r="B15" s="1">
         <v>13</v>
@@ -663,8 +747,10 @@
         <v>15</v>
       </c>
       <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
       <c r="B16" s="1">
         <v>14</v>
@@ -673,8 +759,10 @@
         <v>20</v>
       </c>
       <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>9</v>
       </c>
@@ -685,8 +773,12 @@
         <v>7</v>
       </c>
       <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" s="1"/>
+      <c r="F17" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="1">
         <v>16</v>
@@ -697,8 +789,21 @@
       <c r="D18" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>16</v>
       </c>
@@ -711,8 +816,21 @@
       <c r="D19" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" s="1"/>
+      <c r="F19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="1">
         <v>18</v>
@@ -721,18 +839,22 @@
         <v>17</v>
       </c>
       <c r="D20" s="1"/>
+      <c r="E20" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:C2"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="D1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>